<commit_message>
racesims: Chennai Navkar spares kept — close trim decision
Thambu confirmed the 3 spare Navkar component sets (₹2,63,199) stay as
inventory. Loan ask stays ₹29,31,810 (₹26,68,611 trim option closed).
Resolved across brief, tracker xlsx (both sheets), and wiki (navkar
quote contradiction, per-rig costing open question, hot, log).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/racesims/Racesims Studio, Chennai/RaceSims-Chennai-Project-Payment-Tracker.xlsx
+++ b/racesims/Racesims Studio, Chennai/RaceSims-Chennai-Project-Payment-Tracker.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="\₹#,##0"/>
     <numFmt numFmtId="165" formatCode="₹#,##0"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -191,6 +191,10 @@
       <i val="1"/>
       <color rgb="00833C00"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="001B7A4F"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="15">
@@ -335,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -449,6 +453,13 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,6 +2182,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57" ht="24" customHeight="1" s="23">
       <c r="A57" s="29" t="inlineStr">
         <is>
@@ -2196,9 +2208,9 @@
       </c>
     </row>
     <row r="58" ht="18" customHeight="1" s="23">
-      <c r="A58" s="33" t="inlineStr">
-        <is>
-          <t>★  ₹2,63,199 embedded in Navkar order as spare components (3× cooler/RAM/SSD, 3× PSU, 2× 3500X + 1× 4000D cabinet) — confirm keep or trim</t>
+      <c r="A58" s="58" t="inlineStr">
+        <is>
+          <t>★  ₹2,63,199 spare components (3× cooler/RAM/SSD, 3× PSU, 2× 3500X + 1× 4000D cabinet) KEPT as inventory — confirmed 2026-07-07. Included in the Navkar PO.</t>
         </is>
       </c>
     </row>
@@ -2304,17 +2316,15 @@
       <c r="D7" s="44" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     (if 3 Navkar spare sets trimmed → loan ask)</t>
-        </is>
-      </c>
-      <c r="C8" s="45" t="n">
-        <v>2668611</v>
-      </c>
-      <c r="D8" s="41" t="inlineStr">
-        <is>
-          <t>Spares = ₹2,63,199; DECISION PENDING</t>
+      <c r="B8" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Spares (₹2,63,199) KEPT as inventory — decided 2026-07-07</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="n"/>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Loan ask stays ₹29,31,810 (not trimmed)</t>
         </is>
       </c>
     </row>

</xml_diff>